<commit_message>
Enforce score half-full path consistency
</commit_message>
<xml_diff>
--- a/data/exports/football-recommendations-latest-2026-05-23.xlsx
+++ b/data/exports/football-recommendations-latest-2026-05-23.xlsx
@@ -100,7 +100,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-23T12:41:13.624Z</t>
+          <t>2026-05-23T12:46:41.873Z</t>
         </is>
       </c>
     </row>
@@ -124,7 +124,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:27.458Z</t>
+          <t>2026-05-23T12:46:32.656Z</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>主2.074 平3.581 客3.211</t>
+          <t>主2.075 平3.581 客3.199</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>主-0.205 平+0.217 客+0.496</t>
+          <t>主-0.206 平+0.217 客+0.508</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>主胜-客胜</t>
+          <t>客胜-客胜</t>
         </is>
       </c>
       <c r="P5">
@@ -901,7 +901,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>主2.454 平3.431 客2.636</t>
+          <t>主2.447 平3.431 客2.641</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>主+0.018 平+0.015 客-0.069</t>
+          <t>主+0.025 平+0.015 客-0.074</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1413,12 +1413,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>主胜-客胜</t>
+          <t>客胜-客胜</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="P9">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>主胜-客胜</t>
+          <t>客胜-客胜</t>
         </is>
       </c>
       <c r="P11">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>主1.467 平4.373 客6.839</t>
+          <t>主1.466 平4.372 客6.839</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>主-0.001 平-0.16 客-0.42</t>
+          <t>主0 平-0.159 客-0.42</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>主1.478 平4.695 客5.778</t>
+          <t>主1.482 平4.687 客5.742</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>主-0.043 平-0.039 客+0.2</t>
+          <t>主-0.047 平-0.031 客+0.236</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="P20">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>主3.251 平3.955 客1.998</t>
+          <t>主3.252 平3.954 客1.997</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>主+0.261 平-0.016 客-0.147</t>
+          <t>主+0.26 平-0.015 客-0.146</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -3033,12 +3033,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>主胜-客胜</t>
+          <t>客胜-客胜</t>
         </is>
       </c>
       <c r="P21">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>主2.011 平3.6 客3.312</t>
+          <t>主2.005 平3.6 客3.312</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>主-0.114 平-0.052 客+0.28</t>
+          <t>主-0.108 平-0.052 客+0.28</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>主胜-客胜</t>
+          <t>客胜-客胜</t>
         </is>
       </c>
       <c r="P26">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>盘0.438 主水1.869 客水1.991</t>
+          <t>盘0.406 主水1.908 客水1.957</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>盘-0.781 主水1.876 客水1.914</t>
+          <t>盘-0.781 主水1.877 客水1.912</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>盘-0.433 主水1.984 客水1.84</t>
+          <t>盘-0.433 主水1.987 客水1.839</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>盘-0.3 主水1.85 客水1.971</t>
+          <t>盘-0.3 主水1.851 客水1.969</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>盘-0.75 主水1.825 客水1.936</t>
+          <t>盘-0.75 主水1.823 客水1.938</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:25.061Z</t>
+          <t>2026-05-23T12:46:30.118Z</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:25.061Z</t>
+          <t>2026-05-23T12:46:30.118Z</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:15.009Z</t>
+          <t>2026-05-23T12:46:19.455Z</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4936,13 +4936,13 @@
         </is>
       </c>
       <c r="H4">
-        <v>2.074</v>
+        <v>2.075</v>
       </c>
       <c r="I4">
         <v>3.581</v>
       </c>
       <c r="J4">
-        <v>3.211</v>
+        <v>3.199</v>
       </c>
       <c r="K4">
         <v>1.869</v>
@@ -4954,22 +4954,22 @@
         <v>3.707</v>
       </c>
       <c r="N4">
-        <v>-0.205</v>
+        <v>-0.206</v>
       </c>
       <c r="O4">
         <v>0.217</v>
       </c>
       <c r="P4">
-        <v>0.496</v>
+        <v>0.508</v>
       </c>
       <c r="Q4">
-        <v>-1.042</v>
+        <v>-1.062</v>
       </c>
       <c r="R4">
-        <v>1.104</v>
+        <v>1.125</v>
       </c>
       <c r="S4">
-        <v>1.518</v>
+        <v>1.498</v>
       </c>
       <c r="T4">
         <v>-1.338</v>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:16.065Z</t>
+          <t>2026-05-23T12:46:20.525Z</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="H5">
-        <v>2.454</v>
+        <v>2.447</v>
       </c>
       <c r="I5">
         <v>3.431</v>
       </c>
       <c r="J5">
-        <v>2.636</v>
+        <v>2.641</v>
       </c>
       <c r="K5">
         <v>2.472</v>
@@ -5054,22 +5054,22 @@
         <v>2.567</v>
       </c>
       <c r="N5">
-        <v>0.018</v>
+        <v>0.025</v>
       </c>
       <c r="O5">
         <v>0.015</v>
       </c>
       <c r="P5">
-        <v>-0.069</v>
+        <v>-0.074</v>
       </c>
       <c r="Q5">
-        <v>-0.523</v>
+        <v>-0.562</v>
       </c>
       <c r="R5">
-        <v>1.094</v>
+        <v>1.139</v>
       </c>
       <c r="S5">
-        <v>1.221</v>
+        <v>1.197</v>
       </c>
       <c r="T5">
         <v>-0.554</v>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-23T12:37:54.468Z</t>
+          <t>2026-05-23T12:46:00.322Z</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-05-23T12:37:54.468Z</t>
+          <t>2026-05-23T12:46:00.322Z</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -5327,7 +5327,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:25.062Z</t>
+          <t>2026-05-23T12:46:30.119Z</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.266Z</t>
+          <t>2026-05-23T12:46:31.397Z</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-05-23T12:37:54.468Z</t>
+          <t>2026-05-23T12:46:00.323Z</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.266Z</t>
+          <t>2026-05-23T12:46:31.397Z</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.267Z</t>
+          <t>2026-05-23T12:46:31.399Z</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.272Z</t>
+          <t>2026-05-23T12:46:31.406Z</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:17.123Z</t>
+          <t>2026-05-23T12:46:21.601Z</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -5936,10 +5936,10 @@
         </is>
       </c>
       <c r="H14">
-        <v>1.467</v>
+        <v>1.466</v>
       </c>
       <c r="I14">
-        <v>4.373</v>
+        <v>4.372</v>
       </c>
       <c r="J14">
         <v>6.839</v>
@@ -5954,10 +5954,10 @@
         <v>6.419</v>
       </c>
       <c r="N14">
-        <v>-0.001</v>
+        <v>0</v>
       </c>
       <c r="O14">
-        <v>-0.16</v>
+        <v>-0.159</v>
       </c>
       <c r="P14">
         <v>-0.42</v>
@@ -5966,10 +5966,10 @@
         <v>-1.792</v>
       </c>
       <c r="R14">
-        <v>0.969</v>
+        <v>0.968</v>
       </c>
       <c r="S14">
-        <v>2.252</v>
+        <v>2.258</v>
       </c>
       <c r="T14">
         <v>-1.769</v>
@@ -6027,7 +6027,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.269Z</t>
+          <t>2026-05-23T12:46:31.402Z</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:18.183Z</t>
+          <t>2026-05-23T12:46:22.675Z</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6136,13 +6136,13 @@
         </is>
       </c>
       <c r="H16">
-        <v>1.478</v>
+        <v>1.482</v>
       </c>
       <c r="I16">
-        <v>4.695</v>
+        <v>4.687</v>
       </c>
       <c r="J16">
-        <v>5.778</v>
+        <v>5.742</v>
       </c>
       <c r="K16">
         <v>1.435</v>
@@ -6154,22 +6154,22 @@
         <v>5.978</v>
       </c>
       <c r="N16">
-        <v>-0.043</v>
+        <v>-0.047</v>
       </c>
       <c r="O16">
-        <v>-0.039</v>
+        <v>-0.031</v>
       </c>
       <c r="P16">
-        <v>0.2</v>
+        <v>0.236</v>
       </c>
       <c r="Q16">
-        <v>-1.715</v>
+        <v>-1.677</v>
       </c>
       <c r="R16">
-        <v>1.034</v>
+        <v>0.998</v>
       </c>
       <c r="S16">
-        <v>1.611</v>
+        <v>1.642</v>
       </c>
       <c r="T16">
         <v>-1.815</v>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.272Z</t>
+          <t>2026-05-23T12:46:31.406Z</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-05-23T12:37:54.469Z</t>
+          <t>2026-05-23T12:46:00.323Z</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.270Z</t>
+          <t>2026-05-23T12:46:31.404Z</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -6527,7 +6527,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:19.244Z</t>
+          <t>2026-05-23T12:46:23.749Z</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -6536,13 +6536,13 @@
         </is>
       </c>
       <c r="H20">
-        <v>3.251</v>
+        <v>3.252</v>
       </c>
       <c r="I20">
-        <v>3.955</v>
+        <v>3.954</v>
       </c>
       <c r="J20">
-        <v>1.998</v>
+        <v>1.997</v>
       </c>
       <c r="K20">
         <v>3.512</v>
@@ -6554,22 +6554,22 @@
         <v>1.851</v>
       </c>
       <c r="N20">
-        <v>0.261</v>
+        <v>0.26</v>
       </c>
       <c r="O20">
-        <v>-0.016</v>
+        <v>-0.015</v>
       </c>
       <c r="P20">
-        <v>-0.147</v>
+        <v>-0.146</v>
       </c>
       <c r="Q20">
         <v>-0.158</v>
       </c>
       <c r="R20">
-        <v>1.223</v>
+        <v>1.215</v>
       </c>
       <c r="S20">
-        <v>1.173</v>
+        <v>1.178</v>
       </c>
       <c r="T20">
         <v>-0.181</v>
@@ -6627,7 +6627,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-05-23T12:37:54.469Z</t>
+          <t>2026-05-23T12:46:00.323Z</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -6727,7 +6727,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:20.310Z</t>
+          <t>2026-05-23T12:46:24.807Z</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -6766,10 +6766,10 @@
         <v>-0.769</v>
       </c>
       <c r="R22">
-        <v>1.043</v>
+        <v>1.045</v>
       </c>
       <c r="S22">
-        <v>1.313</v>
+        <v>1.312</v>
       </c>
       <c r="T22">
         <v>-0.754</v>
@@ -6827,7 +6827,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:21.369Z</t>
+          <t>2026-05-23T12:46:26.413Z</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -6866,10 +6866,10 @@
         <v>-0.973</v>
       </c>
       <c r="R23">
-        <v>0.978</v>
+        <v>0.979</v>
       </c>
       <c r="S23">
-        <v>1.435</v>
+        <v>1.434</v>
       </c>
       <c r="T23">
         <v>-0.95</v>
@@ -6927,7 +6927,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:22.426Z</t>
+          <t>2026-05-23T12:46:27.520Z</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -6936,7 +6936,7 @@
         </is>
       </c>
       <c r="H24">
-        <v>2.011</v>
+        <v>2.005</v>
       </c>
       <c r="I24">
         <v>3.6</v>
@@ -6954,7 +6954,7 @@
         <v>3.592</v>
       </c>
       <c r="N24">
-        <v>-0.114</v>
+        <v>-0.108</v>
       </c>
       <c r="O24">
         <v>-0.052</v>
@@ -7027,7 +7027,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.764Z</t>
+          <t>2026-05-23T12:46:31.905Z</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7127,7 +7127,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:23.490Z</t>
+          <t>2026-05-23T12:46:28.577Z</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:25.062Z</t>
+          <t>2026-05-23T12:46:30.120Z</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7236,13 +7236,13 @@
         </is>
       </c>
       <c r="H27">
-        <v>1.371</v>
+        <v>1.369</v>
       </c>
       <c r="I27">
         <v>5.628</v>
       </c>
       <c r="J27">
-        <v>6.385</v>
+        <v>6.396</v>
       </c>
       <c r="K27">
         <v>1.356</v>
@@ -7254,13 +7254,13 @@
         <v>6.568</v>
       </c>
       <c r="N27">
-        <v>-0.015</v>
+        <v>-0.013</v>
       </c>
       <c r="O27">
         <v>-0.374</v>
       </c>
       <c r="P27">
-        <v>0.183</v>
+        <v>0.172</v>
       </c>
       <c r="Q27">
         <v>0.5</v>
@@ -7339,7 +7339,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:42.000Z</t>
+          <t>2026-05-23T12:43:02.000Z</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7348,13 +7348,13 @@
         </is>
       </c>
       <c r="H28">
-        <v>3.485</v>
+        <v>3.453</v>
       </c>
       <c r="I28">
-        <v>3.611</v>
+        <v>3.596</v>
       </c>
       <c r="J28">
-        <v>2.027</v>
+        <v>2.045</v>
       </c>
       <c r="K28">
         <v>3.709</v>
@@ -7366,13 +7366,13 @@
         <v>1.883</v>
       </c>
       <c r="N28">
-        <v>0.224</v>
+        <v>0.256</v>
       </c>
       <c r="O28">
-        <v>0.244</v>
+        <v>0.259</v>
       </c>
       <c r="P28">
-        <v>-0.144</v>
+        <v>-0.162</v>
       </c>
       <c r="Q28">
         <v>0.516</v>
@@ -7384,13 +7384,13 @@
         <v>1.896</v>
       </c>
       <c r="T28">
-        <v>0.438</v>
+        <v>0.406</v>
       </c>
       <c r="U28">
-        <v>1.869</v>
+        <v>1.908</v>
       </c>
       <c r="V28">
-        <v>1.991</v>
+        <v>1.957</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
@@ -7451,7 +7451,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:49.000Z</t>
+          <t>2026-05-23T12:43:10.000Z</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7499,10 +7499,10 @@
         <v>-0.781</v>
       </c>
       <c r="U29">
-        <v>1.876</v>
+        <v>1.877</v>
       </c>
       <c r="V29">
-        <v>1.914</v>
+        <v>1.912</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
@@ -7563,7 +7563,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:50.000Z</t>
+          <t>2026-05-23T12:43:11.000Z</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7572,13 +7572,13 @@
         </is>
       </c>
       <c r="H30">
-        <v>1.936</v>
+        <v>1.937</v>
       </c>
       <c r="I30">
-        <v>3.462</v>
+        <v>3.46</v>
       </c>
       <c r="J30">
-        <v>4.009</v>
+        <v>4.006</v>
       </c>
       <c r="K30">
         <v>1.89</v>
@@ -7590,13 +7590,13 @@
         <v>3.912</v>
       </c>
       <c r="N30">
-        <v>-0.046</v>
+        <v>-0.047</v>
       </c>
       <c r="O30">
-        <v>0.048</v>
+        <v>0.05</v>
       </c>
       <c r="P30">
-        <v>-0.097</v>
+        <v>-0.094</v>
       </c>
       <c r="Q30">
         <v>-0.531</v>
@@ -7675,7 +7675,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-05-23T12:38:26.269Z</t>
+          <t>2026-05-23T12:46:31.401Z</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7787,7 +7787,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:50.000Z</t>
+          <t>2026-05-23T12:43:11.000Z</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:50.000Z</t>
+          <t>2026-05-23T12:43:11.000Z</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:32.000Z</t>
+          <t>2026-05-23T12:42:52.000Z</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:18.000Z</t>
+          <t>2026-05-23T12:42:38.000Z</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8132,13 +8132,13 @@
         </is>
       </c>
       <c r="H35">
-        <v>2.069</v>
+        <v>2.064</v>
       </c>
       <c r="I35">
-        <v>3.387</v>
+        <v>3.392</v>
       </c>
       <c r="J35">
-        <v>3.369</v>
+        <v>3.377</v>
       </c>
       <c r="K35">
         <v>2.112</v>
@@ -8150,13 +8150,13 @@
         <v>3.16</v>
       </c>
       <c r="N35">
-        <v>0.043</v>
+        <v>0.048</v>
       </c>
       <c r="O35">
-        <v>-0.027</v>
+        <v>-0.032</v>
       </c>
       <c r="P35">
-        <v>-0.209</v>
+        <v>-0.217</v>
       </c>
       <c r="Q35">
         <v>-0.267</v>
@@ -8171,10 +8171,10 @@
         <v>-0.433</v>
       </c>
       <c r="U35">
-        <v>1.984</v>
+        <v>1.987</v>
       </c>
       <c r="V35">
-        <v>1.84</v>
+        <v>1.839</v>
       </c>
       <c r="W35" t="inlineStr">
         <is>
@@ -8235,7 +8235,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:18.000Z</t>
+          <t>2026-05-23T12:42:38.000Z</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8244,13 +8244,13 @@
         </is>
       </c>
       <c r="H36">
-        <v>1.921</v>
+        <v>1.92</v>
       </c>
       <c r="I36">
-        <v>3.321</v>
+        <v>3.318</v>
       </c>
       <c r="J36">
-        <v>3.932</v>
+        <v>3.934</v>
       </c>
       <c r="K36">
         <v>2.067</v>
@@ -8262,13 +8262,13 @@
         <v>3.474</v>
       </c>
       <c r="N36">
-        <v>0.146</v>
+        <v>0.147</v>
       </c>
       <c r="O36">
-        <v>-0.164</v>
+        <v>-0.161</v>
       </c>
       <c r="P36">
-        <v>-0.458</v>
+        <v>-0.46</v>
       </c>
       <c r="Q36">
         <v>-0.406</v>
@@ -8347,7 +8347,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:26.000Z</t>
+          <t>2026-05-23T12:42:45.000Z</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8356,13 +8356,13 @@
         </is>
       </c>
       <c r="H37">
-        <v>2.023</v>
+        <v>2.025</v>
       </c>
       <c r="I37">
-        <v>3.57</v>
+        <v>3.567</v>
       </c>
       <c r="J37">
-        <v>3.274</v>
+        <v>3.271</v>
       </c>
       <c r="K37">
         <v>1.778</v>
@@ -8374,13 +8374,13 @@
         <v>3.89</v>
       </c>
       <c r="N37">
-        <v>-0.245</v>
+        <v>-0.247</v>
       </c>
       <c r="O37">
-        <v>0.277</v>
+        <v>0.28</v>
       </c>
       <c r="P37">
-        <v>0.616</v>
+        <v>0.619</v>
       </c>
       <c r="Q37">
         <v>-0.583</v>
@@ -8395,10 +8395,10 @@
         <v>-0.3</v>
       </c>
       <c r="U37">
-        <v>1.85</v>
+        <v>1.851</v>
       </c>
       <c r="V37">
-        <v>1.971</v>
+        <v>1.969</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
@@ -8459,7 +8459,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:27.000Z</t>
+          <t>2026-05-23T12:42:46.000Z</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:27.000Z</t>
+          <t>2026-05-23T12:42:46.000Z</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8583,7 +8583,7 @@
         <v>1.615</v>
       </c>
       <c r="I39">
-        <v>3.748</v>
+        <v>3.744</v>
       </c>
       <c r="J39">
         <v>5.205</v>
@@ -8601,7 +8601,7 @@
         <v>-0.024</v>
       </c>
       <c r="O39">
-        <v>0.02</v>
+        <v>0.024</v>
       </c>
       <c r="P39">
         <v>-0.142</v>
@@ -8619,10 +8619,10 @@
         <v>-0.75</v>
       </c>
       <c r="U39">
-        <v>1.825</v>
+        <v>1.823</v>
       </c>
       <c r="V39">
-        <v>1.936</v>
+        <v>1.938</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
@@ -8683,7 +8683,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-05-23T12:36:27.000Z</t>
+          <t>2026-05-23T12:42:46.000Z</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">

</xml_diff>

<commit_message>
Refresh fused factor recommendation outputs
</commit_message>
<xml_diff>
--- a/data/exports/football-recommendations-latest-2026-05-23.xlsx
+++ b/data/exports/football-recommendations-latest-2026-05-23.xlsx
@@ -101,7 +101,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:34.980Z</t>
+          <t>2026-05-23T13:26:53.325Z</t>
         </is>
       </c>
     </row>
@@ -125,7 +125,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:25.649Z</t>
+          <t>2026-05-23T13:26:44.214Z</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>主2.116 平3.556 客3.122</t>
+          <t>主2.12 平3.556 客3.113</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>主-0.247 平+0.242 客+0.585</t>
+          <t>主-0.251 平+0.242 客+0.594</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
+          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>主2.416 平3.451 客2.675</t>
+          <t>主2.416 平3.445 客2.675</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>主+0.056 平-0.005 客-0.108</t>
+          <t>主+0.056 平+0.001 客-0.108</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.04）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.04）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.88）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.88）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="P6">
-        <v>43.94</v>
+        <v>48.14</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>中高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1366,11 +1366,11 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>平局-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="P7">
-        <v>39.07</v>
+        <v>43.27</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.97）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.97）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.71）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.71）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>主2.62 平3.6 客2.13</t>
+          <t>主2.7 平3.45 客2.13</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>主+0.11 平+0.1 客-0.12</t>
+          <t>主+0.19 平-0.05 客-0.12</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化0</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
@@ -2129,12 +2129,12 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化0</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="P13">
-        <v>31.71</v>
+        <v>35.91</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.66）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.66）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>主1.484 平4.669 客5.713</t>
+          <t>主1.483 平4.672 客5.722</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>主-0.049 平-0.013 客+0.265</t>
+          <t>主-0.048 平-0.016 客+0.256</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.14）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.14）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH14" t="inlineStr">
@@ -2711,12 +2711,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="P15">
-        <v>16.66</v>
+        <v>20.86</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：中高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.57）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.57）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH15" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.83）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.83）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH16" t="inlineStr">
@@ -3061,16 +3061,16 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>平局-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>主胜-平局</t>
+          <t>平局-平局</t>
         </is>
       </c>
       <c r="P17">
-        <v>26.77</v>
+        <v>30.97</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH17" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
+          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
         </is>
       </c>
       <c r="AH18" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH19" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.01）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.01）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH20" t="inlineStr">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH21" t="inlineStr">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.76）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.76）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH22" t="inlineStr">
@@ -4071,26 +4071,26 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>平局-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>主胜-平局</t>
+          <t>平局-平局</t>
         </is>
       </c>
       <c r="P23">
-        <v>61.06</v>
+        <v>65.26</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.85）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.85）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH23" t="inlineStr">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.08）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.08）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH24" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>盘0.5 主水2.02 客水1.82</t>
+          <t>盘-1.516 主水1.964 客水1.879</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>盘0.313 主水1.944 客水1.918</t>
+          <t>盘0.313 主水1.949 客水1.909</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="G4">
-        <v>39.07</v>
+        <v>43.27</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>盘-0.719 主水1.892 客水1.954</t>
+          <t>盘-0.719 主水1.895 客水1.951</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>盘-0.5 主水1.98 客水1.88</t>
+          <t>盘-0.047 主水1.821 客水1.989</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -4695,7 +4695,7 @@
         </is>
       </c>
       <c r="G7">
-        <v>16.66</v>
+        <v>20.86</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>盘-0.5 主水2.1 客水1.7</t>
+          <t>盘-0.483 主水1.999 客水1.837</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>盘-0.75 主水2.1 客水1.7</t>
+          <t>盘-0.5 主水1.904 客水1.86</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>盘-0.283 主水1.877 客水1.94</t>
+          <t>盘-0.283 主水1.878 客水1.94</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>盘-0.969 主水1.895 客水1.865</t>
+          <t>盘-0.969 主水1.889 客水1.871</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>盘0 主水1.818 客水1.947</t>
+          <t>盘0 主水1.819 客水1.946</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
+          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.04）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.04）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.88）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.88）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5615,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="J6">
-        <v>43.94</v>
+        <v>48.14</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="J7">
-        <v>39.07</v>
+        <v>43.27</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -5753,7 +5753,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.97）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.97）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5933,7 +5933,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.71）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.71）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6018,12 +6018,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化0</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6108,12 +6108,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化0</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6203,7 +6203,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6254,7 +6254,7 @@
         </is>
       </c>
       <c r="J13">
-        <v>31.71</v>
+        <v>35.91</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.66）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.66）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.14）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.14）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -6434,7 +6434,7 @@
         </is>
       </c>
       <c r="J15">
-        <v>16.66</v>
+        <v>20.86</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：中高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.57）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.57）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6563,7 +6563,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.83）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.83）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6610,11 +6610,11 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>平局-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="J17">
-        <v>26.77</v>
+        <v>30.97</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -6653,7 +6653,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
+          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
         </is>
       </c>
     </row>
@@ -6833,7 +6833,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.01）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.01）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7013,7 +7013,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.78）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.76）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.76）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7145,16 +7145,16 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>平局-主胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="J23">
-        <v>61.06</v>
+        <v>65.26</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -7193,7 +7193,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.85）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.85）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.08）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.67）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.08）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7368,12 +7368,12 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化0</t>
+          <t>常规｜赔率变化平稳；亚盘变化+0.02</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.95）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.95）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7463,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.2）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.2）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7514,7 +7514,7 @@
         </is>
       </c>
       <c r="J27">
-        <v>39.07</v>
+        <v>43.27</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -7553,7 +7553,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>主判断：客胜，防主胜；冷门：低（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.91）；赔率：首选热度走弱（首选热度走弱；亚盘变化+0.34）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：客胜，防主胜；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.91）；赔率：首选热度走弱（首选热度走弱；亚盘变化+0.34）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7643,7 +7643,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7728,12 +7728,12 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>常规｜资金/赔率支持首选；亚盘变化0</t>
+          <t>常规｜资金/赔率支持首选；亚盘变化+0.2</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.62）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.62）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化+0.2）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
         </is>
       </c>
       <c r="J30">
-        <v>16.66</v>
+        <v>20.86</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.80）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.80）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7913,7 +7913,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化+0.13）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，支撑大于风险</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化+0.13）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，支撑大于风险</t>
         </is>
       </c>
     </row>
@@ -8003,7 +8003,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.66）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.19）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.66）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.19）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8088,12 +8088,12 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>常规｜首选热度走弱；亚盘变化0</t>
+          <t>常规｜首选热度走弱；亚盘变化-0.22</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：低（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.22）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8178,12 +8178,12 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>常规｜首选热度走弱；亚盘变化0</t>
+          <t>常规｜首选热度走弱；亚盘变化-0.09</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.09）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8273,7 +8273,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.81）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化+0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.81）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化+0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8363,7 +8363,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8453,7 +8453,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.87）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.09）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.87）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.09）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8543,7 +8543,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：undefined（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.09）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.09）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:11.619Z</t>
+          <t>2026-05-23T13:26:32.717Z</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -8764,13 +8764,13 @@
         </is>
       </c>
       <c r="H2">
-        <v>2.116</v>
+        <v>2.12</v>
       </c>
       <c r="I2">
         <v>3.556</v>
       </c>
       <c r="J2">
-        <v>3.122</v>
+        <v>3.113</v>
       </c>
       <c r="K2">
         <v>1.869</v>
@@ -8782,22 +8782,22 @@
         <v>3.707</v>
       </c>
       <c r="N2">
-        <v>-0.247</v>
+        <v>-0.251</v>
       </c>
       <c r="O2">
         <v>0.242</v>
       </c>
       <c r="P2">
-        <v>0.585</v>
+        <v>0.594</v>
       </c>
       <c r="Q2">
         <v>-1.042</v>
       </c>
       <c r="R2">
-        <v>1.143</v>
+        <v>1.145</v>
       </c>
       <c r="S2">
-        <v>1.458</v>
+        <v>1.456</v>
       </c>
       <c r="T2">
         <v>-1.338</v>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:12.681Z</t>
+          <t>2026-05-23T13:26:33.829Z</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -8867,7 +8867,7 @@
         <v>2.416</v>
       </c>
       <c r="I3">
-        <v>3.451</v>
+        <v>3.445</v>
       </c>
       <c r="J3">
         <v>2.675</v>
@@ -8885,7 +8885,7 @@
         <v>0.056</v>
       </c>
       <c r="O3">
-        <v>-0.005</v>
+        <v>0.001</v>
       </c>
       <c r="P3">
         <v>-0.108</v>
@@ -8955,7 +8955,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-23T13:23:52.911Z</t>
+          <t>2026-05-23T13:26:11.182Z</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-23T13:23:52.911Z</t>
+          <t>2026-05-23T13:26:11.182Z</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -9155,12 +9155,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:22.192Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84943.html</t>
+          <t>中国体彩网竞彩足球计算器</t>
         </is>
       </c>
       <c r="H6">
@@ -9255,12 +9255,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.653Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84816.html</t>
+          <t>中国体彩网竞彩足球计算器</t>
         </is>
       </c>
       <c r="H7">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-05-23T13:23:52.911Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -9455,12 +9455,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.654Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml+CubeGoal public match filter API https://www.cubegoal.com/odds/84926.html</t>
+          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml</t>
         </is>
       </c>
       <c r="H9">
@@ -9494,19 +9494,19 @@
         <v>-0.25</v>
       </c>
       <c r="R9">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
       <c r="S9">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="T9">
         <v>-0.25</v>
       </c>
       <c r="U9">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
       <c r="V9">
-        <v>1.85</v>
+        <v>1.93</v>
       </c>
       <c r="W9">
         <v>4.15</v>
@@ -9555,12 +9555,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.655Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml+CubeGoal public match filter API https://www.cubegoal.com/odds/84813.html</t>
+          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml</t>
         </is>
       </c>
       <c r="H10">
@@ -9594,19 +9594,19 @@
         <v>-0.75</v>
       </c>
       <c r="R10">
-        <v>1.92</v>
+        <v>1.85</v>
       </c>
       <c r="S10">
-        <v>1.92</v>
+        <v>2</v>
       </c>
       <c r="T10">
-        <v>-0.75</v>
+        <v>-1</v>
       </c>
       <c r="U10">
-        <v>1.92</v>
+        <v>1.94</v>
       </c>
       <c r="V10">
-        <v>1.92</v>
+        <v>1.9</v>
       </c>
       <c r="W10">
         <v>2.51</v>
@@ -9618,10 +9618,10 @@
         <v>2.25</v>
       </c>
       <c r="Z10">
-        <v>2.62</v>
+        <v>2.7</v>
       </c>
       <c r="AA10">
-        <v>3.6</v>
+        <v>3.45</v>
       </c>
       <c r="AB10">
         <v>2.13</v>
@@ -9655,12 +9655,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.660Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml+CubeGoal public match filter API https://www.cubegoal.com/odds/84831.html</t>
+          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml</t>
         </is>
       </c>
       <c r="H11">
@@ -9691,22 +9691,22 @@
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>-0.75</v>
+        <v>-0.5</v>
       </c>
       <c r="R11">
-        <v>2.05</v>
+        <v>1.78</v>
       </c>
       <c r="S11">
-        <v>1.8</v>
+        <v>2.07</v>
       </c>
       <c r="T11">
         <v>-0.75</v>
       </c>
       <c r="U11">
-        <v>2.05</v>
+        <v>2.02</v>
       </c>
       <c r="V11">
-        <v>1.8</v>
+        <v>1.82</v>
       </c>
       <c r="W11">
         <v>3.15</v>
@@ -9755,7 +9755,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:13.746Z</t>
+          <t>2026-05-23T13:26:34.946Z</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -9855,12 +9855,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.657Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84826.html</t>
+          <t>中国体彩网竞彩足球计算器</t>
         </is>
       </c>
       <c r="H13">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:14.818Z</t>
+          <t>2026-05-23T13:26:36.063Z</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -9964,13 +9964,13 @@
         </is>
       </c>
       <c r="H14">
-        <v>1.484</v>
+        <v>1.483</v>
       </c>
       <c r="I14">
-        <v>4.669</v>
+        <v>4.672</v>
       </c>
       <c r="J14">
-        <v>5.713</v>
+        <v>5.722</v>
       </c>
       <c r="K14">
         <v>1.435</v>
@@ -9982,22 +9982,22 @@
         <v>5.978</v>
       </c>
       <c r="N14">
-        <v>-0.049</v>
+        <v>-0.048</v>
       </c>
       <c r="O14">
-        <v>-0.013</v>
+        <v>-0.016</v>
       </c>
       <c r="P14">
-        <v>0.265</v>
+        <v>0.256</v>
       </c>
       <c r="Q14">
         <v>-1.677</v>
       </c>
       <c r="R14">
-        <v>1.008</v>
+        <v>1.007</v>
       </c>
       <c r="S14">
-        <v>1.638</v>
+        <v>1.642</v>
       </c>
       <c r="T14">
         <v>-1.815</v>
@@ -10055,12 +10055,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.660Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84830.html</t>
+          <t>中国体彩网竞彩足球计算器</t>
         </is>
       </c>
       <c r="H15">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-05-23T13:23:52.912Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -10255,12 +10255,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.659Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84828.html</t>
+          <t>中国体彩网竞彩足球计算器</t>
         </is>
       </c>
       <c r="H17">
@@ -10355,7 +10355,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:15.902Z</t>
+          <t>2026-05-23T13:26:37.158Z</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-05-23T13:23:52.912Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -10555,7 +10555,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:16.972Z</t>
+          <t>2026-05-23T13:26:38.269Z</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:18.054Z</t>
+          <t>2026-05-23T13:26:39.391Z</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -10755,7 +10755,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:19.138Z</t>
+          <t>2026-05-23T13:26:40.502Z</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -10855,12 +10855,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:24.695Z</t>
+          <t>2026-05-23T13:26:11.183Z</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84844.html</t>
+          <t>中国体彩网竞彩足球计算器</t>
         </is>
       </c>
       <c r="H23">
@@ -10955,7 +10955,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:20.208Z</t>
+          <t>2026-05-23T13:26:41.586Z</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -11091,22 +11091,22 @@
         <v>0.156</v>
       </c>
       <c r="Q25">
-        <v>0.5</v>
+        <v>-1.531</v>
       </c>
       <c r="R25">
-        <v>2.02</v>
+        <v>1.906</v>
       </c>
       <c r="S25">
-        <v>1.82</v>
+        <v>1.906</v>
       </c>
       <c r="T25">
-        <v>0.5</v>
+        <v>-1.516</v>
       </c>
       <c r="U25">
-        <v>2.02</v>
+        <v>1.964</v>
       </c>
       <c r="V25">
-        <v>1.82</v>
+        <v>1.879</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
@@ -11167,7 +11167,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-05-23T13:22:05.000Z</t>
+          <t>2026-05-23T13:25:23.000Z</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -11215,10 +11215,10 @@
         <v>0.313</v>
       </c>
       <c r="U26">
-        <v>1.944</v>
+        <v>1.949</v>
       </c>
       <c r="V26">
-        <v>1.918</v>
+        <v>1.909</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
@@ -11279,7 +11279,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-05-23T13:22:13.000Z</t>
+          <t>2026-05-23T13:25:30.000Z</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -11327,10 +11327,10 @@
         <v>-0.719</v>
       </c>
       <c r="U27">
-        <v>1.892</v>
+        <v>1.895</v>
       </c>
       <c r="V27">
-        <v>1.954</v>
+        <v>1.951</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
@@ -11391,7 +11391,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-05-23T13:22:14.000Z</t>
+          <t>2026-05-23T13:25:31.000Z</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -11503,7 +11503,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:23.656Z</t>
+          <t>2026-05-23T13:25:31.000Z</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -11539,22 +11539,22 @@
         <v>0.343</v>
       </c>
       <c r="Q29">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="R29">
-        <v>1.98</v>
+        <v>1.879</v>
       </c>
       <c r="S29">
-        <v>1.88</v>
+        <v>1.795</v>
       </c>
       <c r="T29">
-        <v>-0.5</v>
+        <v>-0.047</v>
       </c>
       <c r="U29">
-        <v>1.98</v>
+        <v>1.821</v>
       </c>
       <c r="V29">
-        <v>1.88</v>
+        <v>1.989</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
@@ -11615,7 +11615,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-05-23T13:22:13.000Z</t>
+          <t>2026-05-23T13:25:31.000Z</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-05-23T13:22:13.000Z</t>
+          <t>2026-05-23T13:25:31.000Z</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -11839,7 +11839,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-05-23T13:21:55.000Z</t>
+          <t>2026-05-23T13:25:14.000Z</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -11951,7 +11951,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:22.192Z</t>
+          <t>2026-05-23T13:25:00.000Z</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -11987,22 +11987,22 @@
         <v>-0.296</v>
       </c>
       <c r="Q33">
-        <v>-0.5</v>
+        <v>-0.267</v>
       </c>
       <c r="R33">
-        <v>2.1</v>
+        <v>1.858</v>
       </c>
       <c r="S33">
-        <v>1.7</v>
+        <v>1.957</v>
       </c>
       <c r="T33">
-        <v>-0.5</v>
+        <v>-0.483</v>
       </c>
       <c r="U33">
-        <v>2.1</v>
+        <v>1.999</v>
       </c>
       <c r="V33">
-        <v>1.7</v>
+        <v>1.837</v>
       </c>
       <c r="W33" t="inlineStr">
         <is>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:22.191Z</t>
+          <t>2026-05-23T13:25:00.000Z</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -12099,22 +12099,22 @@
         <v>-0.534</v>
       </c>
       <c r="Q34">
-        <v>-0.75</v>
+        <v>-0.406</v>
       </c>
       <c r="R34">
-        <v>2.1</v>
+        <v>1.936</v>
       </c>
       <c r="S34">
-        <v>1.7</v>
+        <v>1.872</v>
       </c>
       <c r="T34">
-        <v>-0.75</v>
+        <v>-0.5</v>
       </c>
       <c r="U34">
-        <v>2.1</v>
+        <v>1.904</v>
       </c>
       <c r="V34">
-        <v>1.7</v>
+        <v>1.86</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-05-23T13:21:48.000Z</t>
+          <t>2026-05-23T13:25:07.000Z</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -12184,7 +12184,7 @@
         </is>
       </c>
       <c r="H35">
-        <v>2.077</v>
+        <v>2.076</v>
       </c>
       <c r="I35">
         <v>3.54</v>
@@ -12202,7 +12202,7 @@
         <v>3.89</v>
       </c>
       <c r="N35">
-        <v>-0.299</v>
+        <v>-0.298</v>
       </c>
       <c r="O35">
         <v>0.307</v>
@@ -12223,7 +12223,7 @@
         <v>-0.283</v>
       </c>
       <c r="U35">
-        <v>1.877</v>
+        <v>1.878</v>
       </c>
       <c r="V35">
         <v>1.94</v>
@@ -12287,7 +12287,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-05-23T13:21:48.000Z</t>
+          <t>2026-05-23T13:25:08.000Z</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-05-23T13:21:49.000Z</t>
+          <t>2026-05-23T13:25:08.000Z</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -12447,10 +12447,10 @@
         <v>-0.969</v>
       </c>
       <c r="U37">
-        <v>1.895</v>
+        <v>1.889</v>
       </c>
       <c r="V37">
-        <v>1.865</v>
+        <v>1.871</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-05-23T13:21:49.000Z</t>
+          <t>2026-05-23T13:25:08.000Z</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -12559,10 +12559,10 @@
         <v>0</v>
       </c>
       <c r="U38">
-        <v>1.818</v>
+        <v>1.819</v>
       </c>
       <c r="V38">
-        <v>1.947</v>
+        <v>1.946</v>
       </c>
       <c r="W38" t="inlineStr">
         <is>
@@ -12899,7 +12899,7 @@
         </is>
       </c>
       <c r="G6">
-        <v>43.94</v>
+        <v>48.14</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -12949,7 +12949,7 @@
         </is>
       </c>
       <c r="G7">
-        <v>39.07</v>
+        <v>43.27</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -13249,7 +13249,7 @@
         </is>
       </c>
       <c r="G13">
-        <v>31.71</v>
+        <v>35.91</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -13349,7 +13349,7 @@
         </is>
       </c>
       <c r="G15">
-        <v>16.66</v>
+        <v>20.86</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -13449,7 +13449,7 @@
         </is>
       </c>
       <c r="G17">
-        <v>26.77</v>
+        <v>30.97</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -13749,7 +13749,7 @@
         </is>
       </c>
       <c r="G23">
-        <v>61.06</v>
+        <v>65.26</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -13949,7 +13949,7 @@
         </is>
       </c>
       <c r="G27">
-        <v>39.07</v>
+        <v>43.27</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -14099,7 +14099,7 @@
         </is>
       </c>
       <c r="G30">
-        <v>16.66</v>
+        <v>20.86</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refresh verified football recommendation table
</commit_message>
<xml_diff>
--- a/data/exports/football-recommendations-latest-2026-05-23.xlsx
+++ b/data/exports/football-recommendations-latest-2026-05-23.xlsx
@@ -101,7 +101,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:53.325Z</t>
+          <t>2026-05-23T14:01:04.359Z</t>
         </is>
       </c>
     </row>
@@ -125,7 +125,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:44.214Z</t>
+          <t>2026-05-23T14:00:54.824Z</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>主2.12 平3.556 客3.113</t>
+          <t>主2.121 平3.547 客3.112</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>主-0.251 平+0.242 客+0.594</t>
+          <t>主-0.252 平+0.251 客+0.595</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -599,12 +599,12 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>常规｜资金/赔率支持首选；亚盘变化-0.3</t>
+          <t>常规｜资金/赔率支持首选；亚盘变化-0.32</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
+          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.32）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>主2.416 平3.445 客2.675</t>
+          <t>主2.394 平3.515 客2.657</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>主+0.056 平+0.001 客-0.108</t>
+          <t>主+0.078 平-0.069 客-0.09</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -769,12 +769,12 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.04</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.03</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.04）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.03）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>主2.6 平3.2 客2.32</t>
+          <t>主2.4 平3.2 客2.5</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>主-0.21 平-0.05 客+0.17</t>
+          <t>主-0.41 平-0.05 客+0.35</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -1166,27 +1166,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>28.4%</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>48.7%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="P6">
-        <v>48.14</v>
+        <v>46.74</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1224,12 +1224,12 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>主3.97 平3.05 客1.82</t>
+          <t>主4.1 平3.12 客1.77</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>主-0.68 平-0.32 客+0.2</t>
+          <t>主-0.55 平-0.25 客+0.15</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1239,12 +1239,12 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>主1.75 平3.42 客3.76</t>
+          <t>主1.79 平3.4 客3.62</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>主-0.23 平+0.04 客+0.71</t>
+          <t>主-0.19 平+0.02 客+0.57</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75</t>
+          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>45.6%</t>
+          <t>44.7%</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1366,11 +1366,11 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>主胜-主胜</t>
+          <t>平局-主胜</t>
         </is>
       </c>
       <c r="P7">
-        <v>43.27</v>
+        <v>36.66</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>主3.05 平3.5 客1.94</t>
+          <t>主2.95 平3.5 客1.98</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>主+0.17 平-0.05 客-0.06</t>
+          <t>主+0.07 平-0.05 客-0.02</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>主1.65 平3.8 客3.85</t>
+          <t>主1.62 平3.85 客4</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>主+0.04 平-0.1 客-0.15</t>
+          <t>主+0.01 平-0.05 客0</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>低｜主方向概率领先</t>
+          <t>低｜备选赔付不高，市场不排除</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74</t>
+          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.73</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防主胜；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.73）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
@@ -1579,12 +1579,12 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>主1.74 平4.25 客3.13</t>
+          <t>主1.7 平4.5 客3.13</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>主-0.11 平+0.25 客+0.18</t>
+          <t>主-0.15 平+0.5 客+0.18</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>主2.7 平3.45 客2.13</t>
+          <t>主2.8 平3.45 客2.08</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>主+0.19 平-0.05 客-0.12</t>
+          <t>主+0.29 平-0.05 客-0.17</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
+          <t>常规｜赔率变化平稳；亚盘变化0</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
@@ -2129,12 +2129,12 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
+          <t>常规｜赔率变化平稳；亚盘变化0</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>主1.462 平4.38 客6.89</t>
+          <t>主1.465 平4.371 客6.835</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>主+0.004 平-0.167 客-0.471</t>
+          <t>主+0.001 平-0.158 客-0.416</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="P13">
-        <v>35.91</v>
+        <v>31.71</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>主1.483 平4.672 客5.722</t>
+          <t>主1.487 平4.655 客5.638</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>主-0.048 平-0.016 客+0.256</t>
+          <t>主-0.052 平+0.001 客+0.34</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -2639,12 +2639,12 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.14</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.18</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.14）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.18）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
       <c r="AH14" t="inlineStr">
@@ -2711,12 +2711,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="P15">
-        <v>20.86</v>
+        <v>16.66</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -3061,16 +3061,16 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>主胜-主胜</t>
+          <t>平局-主胜</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>平局-平局</t>
+          <t>主胜-平局</t>
         </is>
       </c>
       <c r="P17">
-        <v>30.97</v>
+        <v>26.77</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>主3.214 平3.926 客2.015</t>
+          <t>主3.236 平3.918 客2.001</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>主+0.298 平+0.013 客-0.164</t>
+          <t>主+0.276 平+0.021 客-0.15</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>主2.11 平3.554 客3.115</t>
+          <t>主2.113 平3.549 客3.111</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>主+0.031 平-0.008 客-0.168</t>
+          <t>主+0.028 平-0.003 客-0.164</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>主1.854 平3.707 客3.745</t>
+          <t>主1.854 平3.713 客3.746</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>主+0.011 平-0.112 客-0.096</t>
+          <t>主+0.011 平-0.118 客-0.097</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>主2.005 平3.6 客3.312</t>
+          <t>主2.005 平3.598 客3.313</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>主-0.108 平-0.052 客+0.28</t>
+          <t>主-0.108 平-0.05 客+0.279</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
@@ -4071,26 +4071,26 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>主胜-主胜</t>
+          <t>平局-主胜</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>平局-平局</t>
+          <t>主胜-平局</t>
         </is>
       </c>
       <c r="P23">
-        <v>65.26</v>
+        <v>61.06</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>主2.389 平3.895 客2.495</t>
+          <t>主2.395 平3.897 客2.495</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>主-0.079 平-0.071 客+0.06</t>
+          <t>主-0.085 平-0.073 客+0.06</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>盘-1.516 主水1.964 客水1.879</t>
+          <t>盘0.5 主水2.02 客水1.82</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>盘0.313 主水1.949 客水1.909</t>
+          <t>盘0.281 主水1.958 客水1.833</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="G4">
-        <v>43.27</v>
+        <v>36.66</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -4560,12 +4560,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>盘-0.719 主水1.895 客水1.951</t>
+          <t>盘-0.719 主水1.918 客水1.929</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>概率差 17%；14场严格定胆规则：未入强胆池，降为覆盖；经模型综合分析：意甲，主胜概率领先平局；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六013 胜平负方向强制一致</t>
+          <t>概率差 15%；14场严格定胆规则：未入强胆池，降为覆盖；经模型综合分析：意甲，主胜概率领先平局；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六013 胜平负方向强制一致</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4656,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>盘-0.047 主水1.821 客水1.989</t>
+          <t>盘-0.5 主水1.98 客水1.88</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -4695,7 +4695,7 @@
         </is>
       </c>
       <c r="G7">
-        <v>20.86</v>
+        <v>16.66</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -4704,7 +4704,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>盘-0.578 主水1.888 客水1.958</t>
+          <t>盘-0.578 主水1.887 客水1.958</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>盘-0.25 主水1.934 客水1.862</t>
+          <t>盘-0.25 主水2.02 客水1.846</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>盘-0.281 主水1.964 客水1.859</t>
+          <t>盘-0.281 主水1.952 客水1.892</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>盘-0.483 主水1.999 客水1.837</t>
+          <t>盘-0.5 主水2.1 客水1.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>盘-0.5 主水1.904 客水1.86</t>
+          <t>盘-0.75 主水2.1 客水1.7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>盘-0.283 主水1.878 客水1.94</t>
+          <t>盘-0.283 主水1.875 客水1.948</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>盘-0.517 主水1.921 客水1.896</t>
+          <t>盘-0.517 主水1.901 客水1.928</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>盘-0.969 主水1.889 客水1.871</t>
+          <t>盘-0.969 主水1.878 客水1.884</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>盘0 主水1.819 客水1.946</t>
+          <t>盘0.016 主水1.804 客水1.964</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -5298,12 +5298,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>常规｜资金/赔率支持首选；亚盘变化-0.3</t>
+          <t>常规｜资金/赔率支持首选；亚盘变化-0.32</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.3）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
+          <t>主判断：主胜，防客胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化-0.32）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，支撑大于风险</t>
         </is>
       </c>
     </row>
@@ -5388,12 +5388,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.04</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.03</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.04）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.64）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.03）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5615,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="J6">
-        <v>48.14</v>
+        <v>46.74</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -5638,7 +5638,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75</t>
+          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.75）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.77）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="J7">
-        <v>43.27</v>
+        <v>36.66</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -5723,12 +5723,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>低｜主方向概率领先</t>
+          <t>低｜备选赔付不高，市场不排除</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74</t>
+          <t>中性｜无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.73</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -5753,7 +5753,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>主判断：客胜，防主胜；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.74）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
+          <t>主判断：客胜，防主胜；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.73）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6018,12 +6018,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
+          <t>常规｜赔率变化平稳；亚盘变化0</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.89）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6108,12 +6108,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.25</t>
+          <t>常规｜赔率变化平稳；亚盘变化0</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.25）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.82）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6254,7 +6254,7 @@
         </is>
       </c>
       <c r="J13">
-        <v>35.91</v>
+        <v>31.71</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -6378,12 +6378,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化-0.14</t>
+          <t>常规｜赔率变化平稳；亚盘变化-0.18</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.14）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.92）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化-0.18）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -6434,7 +6434,7 @@
         </is>
       </c>
       <c r="J15">
-        <v>20.86</v>
+        <v>16.66</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -6610,11 +6610,11 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>主胜-主胜</t>
+          <t>平局-主胜</t>
         </is>
       </c>
       <c r="J17">
-        <v>30.97</v>
+        <v>26.77</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -7145,16 +7145,16 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>主胜-主胜</t>
+          <t>平局-主胜</t>
         </is>
       </c>
       <c r="J23">
-        <v>65.26</v>
+        <v>61.06</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -7368,12 +7368,12 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化+0.02</t>
+          <t>常规｜赔率变化平稳；亚盘变化0</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.95）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.02）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（主方向概率领先）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.95）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7458,12 +7458,12 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>常规｜首选热度走弱；亚盘变化-0.2</t>
+          <t>常规｜首选热度走弱；亚盘变化-0.23</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.2）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.79）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.23）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7514,7 +7514,7 @@
         </is>
       </c>
       <c r="J27">
-        <v>43.27</v>
+        <v>36.66</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -7728,12 +7728,12 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>常规｜资金/赔率支持首选；亚盘变化+0.2</t>
+          <t>常规｜资金/赔率支持首选；亚盘变化0</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.62）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化+0.2）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.62）；赔率：资金/赔率支持首选（资金/赔率支持首选；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：中强信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
         </is>
       </c>
       <c r="J30">
-        <v>20.86</v>
+        <v>16.66</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -8088,12 +8088,12 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>常规｜首选热度走弱；亚盘变化-0.22</t>
+          <t>常规｜首选热度走弱；亚盘变化0</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.22）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8178,12 +8178,12 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>常规｜首选热度走弱；亚盘变化-0.09</t>
+          <t>常规｜首选热度走弱；亚盘变化0</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化-0.09）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防平局；冷门：低（备选赔付不高，市场不排除）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.70）；赔率：首选热度走弱（首选热度走弱；亚盘变化0）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8538,12 +8538,12 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>常规｜赔率变化平稳；亚盘变化+0.09</t>
+          <t>常规｜赔率变化平稳；亚盘变化+0.11</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.09）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
+          <t>主判断：主胜，防客胜；冷门：中高（概率差过小）；大小球：中性（无明确大小球盘口，使用比分/蒙特卡洛推导，模型总进球2.63）；赔率：赔率变化平稳（赔率变化平稳；亚盘变化+0.11）；状态/阵容：近期状态源未完全匹配；未匹配预计/实际阵容，临场需复核；综合：谨慎信心，风险需覆盖</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:32.717Z</t>
+          <t>2026-05-23T14:00:42.575Z</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -8764,13 +8764,13 @@
         </is>
       </c>
       <c r="H2">
-        <v>2.12</v>
+        <v>2.121</v>
       </c>
       <c r="I2">
-        <v>3.556</v>
+        <v>3.547</v>
       </c>
       <c r="J2">
-        <v>3.113</v>
+        <v>3.112</v>
       </c>
       <c r="K2">
         <v>1.869</v>
@@ -8782,22 +8782,22 @@
         <v>3.707</v>
       </c>
       <c r="N2">
-        <v>-0.251</v>
+        <v>-0.252</v>
       </c>
       <c r="O2">
-        <v>0.242</v>
+        <v>0.251</v>
       </c>
       <c r="P2">
-        <v>0.594</v>
+        <v>0.595</v>
       </c>
       <c r="Q2">
-        <v>-1.042</v>
+        <v>-1.019</v>
       </c>
       <c r="R2">
-        <v>1.145</v>
+        <v>1.138</v>
       </c>
       <c r="S2">
-        <v>1.456</v>
+        <v>1.448</v>
       </c>
       <c r="T2">
         <v>-1.338</v>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:33.829Z</t>
+          <t>2026-05-23T14:00:43.640Z</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -8864,13 +8864,13 @@
         </is>
       </c>
       <c r="H3">
-        <v>2.416</v>
+        <v>2.394</v>
       </c>
       <c r="I3">
-        <v>3.445</v>
+        <v>3.515</v>
       </c>
       <c r="J3">
-        <v>2.675</v>
+        <v>2.657</v>
       </c>
       <c r="K3">
         <v>2.472</v>
@@ -8882,22 +8882,22 @@
         <v>2.567</v>
       </c>
       <c r="N3">
-        <v>0.056</v>
+        <v>0.078</v>
       </c>
       <c r="O3">
-        <v>0.001</v>
+        <v>-0.069</v>
       </c>
       <c r="P3">
-        <v>-0.108</v>
+        <v>-0.09</v>
       </c>
       <c r="Q3">
-        <v>-0.512</v>
+        <v>-0.523</v>
       </c>
       <c r="R3">
-        <v>1.046</v>
+        <v>1.033</v>
       </c>
       <c r="S3">
-        <v>1.275</v>
+        <v>1.285</v>
       </c>
       <c r="T3">
         <v>-0.554</v>
@@ -8955,7 +8955,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.182Z</t>
+          <t>2026-05-23T14:00:20.622Z</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -9018,13 +9018,13 @@
         <v>2.15</v>
       </c>
       <c r="Z4">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="AA4">
         <v>3.2</v>
       </c>
       <c r="AB4">
-        <v>2.32</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="5">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.182Z</t>
+          <t>2026-05-23T14:00:20.622Z</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -9155,12 +9155,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:52.590Z</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器</t>
+          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84943.html</t>
         </is>
       </c>
       <c r="H6">
@@ -9173,22 +9173,22 @@
         <v>1.62</v>
       </c>
       <c r="K6">
-        <v>3.97</v>
+        <v>4.1</v>
       </c>
       <c r="L6">
-        <v>3.05</v>
+        <v>3.12</v>
       </c>
       <c r="M6">
-        <v>1.82</v>
+        <v>1.77</v>
       </c>
       <c r="N6">
-        <v>-0.68</v>
+        <v>-0.55</v>
       </c>
       <c r="O6">
-        <v>-0.32</v>
+        <v>-0.25</v>
       </c>
       <c r="P6">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="Q6">
         <v>0.5</v>
@@ -9218,13 +9218,13 @@
         <v>3.05</v>
       </c>
       <c r="Z6">
-        <v>1.75</v>
+        <v>1.79</v>
       </c>
       <c r="AA6">
-        <v>3.42</v>
+        <v>3.4</v>
       </c>
       <c r="AB6">
-        <v>3.76</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="7">
@@ -9255,12 +9255,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:53.678Z</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器</t>
+          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84816.html</t>
         </is>
       </c>
       <c r="H7">
@@ -9273,22 +9273,22 @@
         <v>2</v>
       </c>
       <c r="K7">
-        <v>3.05</v>
+        <v>2.95</v>
       </c>
       <c r="L7">
         <v>3.5</v>
       </c>
       <c r="M7">
-        <v>1.94</v>
+        <v>1.98</v>
       </c>
       <c r="N7">
-        <v>0.17</v>
+        <v>0.07</v>
       </c>
       <c r="O7">
         <v>-0.05</v>
       </c>
       <c r="P7">
-        <v>-0.06</v>
+        <v>-0.02</v>
       </c>
       <c r="Q7">
         <v>0.25</v>
@@ -9318,13 +9318,13 @@
         <v>4</v>
       </c>
       <c r="Z7">
-        <v>1.65</v>
+        <v>1.62</v>
       </c>
       <c r="AA7">
-        <v>3.8</v>
+        <v>3.85</v>
       </c>
       <c r="AB7">
-        <v>3.85</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:20.622Z</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -9418,10 +9418,10 @@
         <v>2.95</v>
       </c>
       <c r="Z8">
-        <v>1.74</v>
+        <v>1.7</v>
       </c>
       <c r="AA8">
-        <v>4.25</v>
+        <v>4.5</v>
       </c>
       <c r="AB8">
         <v>3.13</v>
@@ -9455,12 +9455,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:53.678Z</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml</t>
+          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml+CubeGoal public match filter API https://www.cubegoal.com/odds/84926.html</t>
         </is>
       </c>
       <c r="H9">
@@ -9494,19 +9494,19 @@
         <v>-0.25</v>
       </c>
       <c r="R9">
+        <v>1.95</v>
+      </c>
+      <c r="S9">
         <v>1.85</v>
-      </c>
-      <c r="S9">
-        <v>2</v>
       </c>
       <c r="T9">
         <v>-0.25</v>
       </c>
       <c r="U9">
+        <v>1.95</v>
+      </c>
+      <c r="V9">
         <v>1.85</v>
-      </c>
-      <c r="V9">
-        <v>1.93</v>
       </c>
       <c r="W9">
         <v>4.15</v>
@@ -9555,12 +9555,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:53.680Z</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml</t>
+          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml+CubeGoal public match filter API https://www.cubegoal.com/odds/84813.html</t>
         </is>
       </c>
       <c r="H10">
@@ -9594,19 +9594,19 @@
         <v>-0.75</v>
       </c>
       <c r="R10">
-        <v>1.85</v>
+        <v>1.92</v>
       </c>
       <c r="S10">
-        <v>2</v>
+        <v>1.92</v>
       </c>
       <c r="T10">
-        <v>-1</v>
+        <v>-0.75</v>
       </c>
       <c r="U10">
-        <v>1.94</v>
+        <v>1.92</v>
       </c>
       <c r="V10">
-        <v>1.9</v>
+        <v>1.92</v>
       </c>
       <c r="W10">
         <v>2.51</v>
@@ -9618,13 +9618,13 @@
         <v>2.25</v>
       </c>
       <c r="Z10">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="AA10">
         <v>3.45</v>
       </c>
       <c r="AB10">
-        <v>2.13</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="11">
@@ -9655,12 +9655,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:53.688Z</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml</t>
+          <t>中国体彩网竞彩足球计算器+Sina euro-asian contrast https://sports.sina.com.cn/l/2026-05-23/doc-inhyvtiw5662178.shtml+CubeGoal public match filter API https://www.cubegoal.com/odds/84831.html</t>
         </is>
       </c>
       <c r="H11">
@@ -9691,22 +9691,22 @@
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>-0.5</v>
+        <v>-0.75</v>
       </c>
       <c r="R11">
-        <v>1.78</v>
+        <v>2.05</v>
       </c>
       <c r="S11">
-        <v>2.07</v>
+        <v>1.8</v>
       </c>
       <c r="T11">
         <v>-0.75</v>
       </c>
       <c r="U11">
-        <v>2.02</v>
+        <v>2.05</v>
       </c>
       <c r="V11">
-        <v>1.82</v>
+        <v>1.8</v>
       </c>
       <c r="W11">
         <v>3.15</v>
@@ -9755,7 +9755,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:34.946Z</t>
+          <t>2026-05-23T14:00:44.708Z</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -9764,13 +9764,13 @@
         </is>
       </c>
       <c r="H12">
-        <v>1.462</v>
+        <v>1.465</v>
       </c>
       <c r="I12">
-        <v>4.38</v>
+        <v>4.371</v>
       </c>
       <c r="J12">
-        <v>6.89</v>
+        <v>6.835</v>
       </c>
       <c r="K12">
         <v>1.466</v>
@@ -9782,22 +9782,22 @@
         <v>6.419</v>
       </c>
       <c r="N12">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="O12">
-        <v>-0.167</v>
+        <v>-0.158</v>
       </c>
       <c r="P12">
-        <v>-0.471</v>
+        <v>-0.416</v>
       </c>
       <c r="Q12">
         <v>-1.792</v>
       </c>
       <c r="R12">
-        <v>0.965</v>
+        <v>0.964</v>
       </c>
       <c r="S12">
-        <v>2.263</v>
+        <v>2.26</v>
       </c>
       <c r="T12">
         <v>-1.769</v>
@@ -9855,12 +9855,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:53.683Z</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器</t>
+          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84826.html</t>
         </is>
       </c>
       <c r="H13">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:36.063Z</t>
+          <t>2026-05-23T14:00:45.772Z</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -9964,13 +9964,13 @@
         </is>
       </c>
       <c r="H14">
-        <v>1.483</v>
+        <v>1.487</v>
       </c>
       <c r="I14">
-        <v>4.672</v>
+        <v>4.655</v>
       </c>
       <c r="J14">
-        <v>5.722</v>
+        <v>5.638</v>
       </c>
       <c r="K14">
         <v>1.435</v>
@@ -9982,22 +9982,22 @@
         <v>5.978</v>
       </c>
       <c r="N14">
-        <v>-0.048</v>
+        <v>-0.052</v>
       </c>
       <c r="O14">
-        <v>-0.016</v>
+        <v>0.001</v>
       </c>
       <c r="P14">
-        <v>0.256</v>
+        <v>0.34</v>
       </c>
       <c r="Q14">
-        <v>-1.677</v>
+        <v>-1.638</v>
       </c>
       <c r="R14">
-        <v>1.007</v>
+        <v>0.985</v>
       </c>
       <c r="S14">
-        <v>1.642</v>
+        <v>1.664</v>
       </c>
       <c r="T14">
         <v>-1.815</v>
@@ -10055,12 +10055,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:53.687Z</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器</t>
+          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84830.html</t>
         </is>
       </c>
       <c r="H15">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:20.623Z</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -10255,12 +10255,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:53.686Z</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器</t>
+          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84828.html</t>
         </is>
       </c>
       <c r="H17">
@@ -10355,7 +10355,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:37.158Z</t>
+          <t>2026-05-23T14:00:46.841Z</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -10364,13 +10364,13 @@
         </is>
       </c>
       <c r="H18">
-        <v>3.214</v>
+        <v>3.236</v>
       </c>
       <c r="I18">
-        <v>3.926</v>
+        <v>3.918</v>
       </c>
       <c r="J18">
-        <v>2.015</v>
+        <v>2.001</v>
       </c>
       <c r="K18">
         <v>3.512</v>
@@ -10382,22 +10382,22 @@
         <v>1.851</v>
       </c>
       <c r="N18">
-        <v>0.298</v>
+        <v>0.276</v>
       </c>
       <c r="O18">
-        <v>0.013</v>
+        <v>0.021</v>
       </c>
       <c r="P18">
-        <v>-0.164</v>
+        <v>-0.15</v>
       </c>
       <c r="Q18">
         <v>-0.158</v>
       </c>
       <c r="R18">
-        <v>1.192</v>
+        <v>1.203</v>
       </c>
       <c r="S18">
-        <v>1.205</v>
+        <v>1.191</v>
       </c>
       <c r="T18">
         <v>-0.181</v>
@@ -10455,7 +10455,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:20.623Z</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -10555,7 +10555,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:38.269Z</t>
+          <t>2026-05-23T14:00:47.901Z</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -10564,13 +10564,13 @@
         </is>
       </c>
       <c r="H20">
-        <v>2.11</v>
+        <v>2.113</v>
       </c>
       <c r="I20">
-        <v>3.554</v>
+        <v>3.549</v>
       </c>
       <c r="J20">
-        <v>3.115</v>
+        <v>3.111</v>
       </c>
       <c r="K20">
         <v>2.141</v>
@@ -10582,22 +10582,22 @@
         <v>2.947</v>
       </c>
       <c r="N20">
-        <v>0.031</v>
+        <v>0.028</v>
       </c>
       <c r="O20">
-        <v>-0.008</v>
+        <v>-0.003</v>
       </c>
       <c r="P20">
-        <v>-0.168</v>
+        <v>-0.164</v>
       </c>
       <c r="Q20">
         <v>-0.762</v>
       </c>
       <c r="R20">
-        <v>1.061</v>
+        <v>1.064</v>
       </c>
       <c r="S20">
-        <v>1.29</v>
+        <v>1.287</v>
       </c>
       <c r="T20">
         <v>-0.754</v>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:39.391Z</t>
+          <t>2026-05-23T14:00:48.959Z</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -10667,10 +10667,10 @@
         <v>1.854</v>
       </c>
       <c r="I21">
-        <v>3.707</v>
+        <v>3.713</v>
       </c>
       <c r="J21">
-        <v>3.745</v>
+        <v>3.746</v>
       </c>
       <c r="K21">
         <v>1.865</v>
@@ -10685,19 +10685,19 @@
         <v>0.011</v>
       </c>
       <c r="O21">
-        <v>-0.112</v>
+        <v>-0.118</v>
       </c>
       <c r="P21">
-        <v>-0.096</v>
+        <v>-0.097</v>
       </c>
       <c r="Q21">
         <v>-0.973</v>
       </c>
       <c r="R21">
-        <v>0.979</v>
+        <v>0.977</v>
       </c>
       <c r="S21">
-        <v>1.434</v>
+        <v>1.436</v>
       </c>
       <c r="T21">
         <v>-0.95</v>
@@ -10755,7 +10755,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:40.502Z</t>
+          <t>2026-05-23T14:00:50.023Z</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -10767,10 +10767,10 @@
         <v>2.005</v>
       </c>
       <c r="I22">
-        <v>3.6</v>
+        <v>3.598</v>
       </c>
       <c r="J22">
-        <v>3.312</v>
+        <v>3.313</v>
       </c>
       <c r="K22">
         <v>1.897</v>
@@ -10785,16 +10785,16 @@
         <v>-0.108</v>
       </c>
       <c r="O22">
-        <v>-0.052</v>
+        <v>-0.05</v>
       </c>
       <c r="P22">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="Q22">
         <v>-0.923</v>
       </c>
       <c r="R22">
-        <v>1.122</v>
+        <v>1.123</v>
       </c>
       <c r="S22">
         <v>1.245</v>
@@ -10855,12 +10855,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:11.183Z</t>
+          <t>2026-05-23T14:00:54.112Z</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>中国体彩网竞彩足球计算器</t>
+          <t>中国体彩网竞彩足球计算器+CubeGoal public match filter API https://www.cubegoal.com/odds/84844.html</t>
         </is>
       </c>
       <c r="H23">
@@ -10955,7 +10955,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-05-23T13:26:41.586Z</t>
+          <t>2026-05-23T14:00:51.078Z</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -10964,10 +10964,10 @@
         </is>
       </c>
       <c r="H24">
-        <v>2.389</v>
+        <v>2.395</v>
       </c>
       <c r="I24">
-        <v>3.895</v>
+        <v>3.897</v>
       </c>
       <c r="J24">
         <v>2.495</v>
@@ -10982,10 +10982,10 @@
         <v>2.555</v>
       </c>
       <c r="N24">
-        <v>-0.079</v>
+        <v>-0.085</v>
       </c>
       <c r="O24">
-        <v>-0.071</v>
+        <v>-0.073</v>
       </c>
       <c r="P24">
         <v>0.06</v>
@@ -10994,10 +10994,10 @@
         <v>-0.585</v>
       </c>
       <c r="R24">
-        <v>1.122</v>
+        <v>1.124</v>
       </c>
       <c r="S24">
-        <v>1.169</v>
+        <v>1.17</v>
       </c>
       <c r="T24">
         <v>-0.662</v>
@@ -11055,7 +11055,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-05-23T13:24:22.193Z</t>
+          <t>2026-05-23T14:00:52.592Z</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -11064,13 +11064,13 @@
         </is>
       </c>
       <c r="H25">
-        <v>1.369</v>
+        <v>1.368</v>
       </c>
       <c r="I25">
-        <v>5.615</v>
+        <v>5.611</v>
       </c>
       <c r="J25">
-        <v>6.412</v>
+        <v>6.415</v>
       </c>
       <c r="K25">
         <v>1.356</v>
@@ -11082,31 +11082,31 @@
         <v>6.568</v>
       </c>
       <c r="N25">
-        <v>-0.013</v>
+        <v>-0.012</v>
       </c>
       <c r="O25">
-        <v>-0.361</v>
+        <v>-0.357</v>
       </c>
       <c r="P25">
-        <v>0.156</v>
+        <v>0.153</v>
       </c>
       <c r="Q25">
-        <v>-1.531</v>
+        <v>0.5</v>
       </c>
       <c r="R25">
-        <v>1.906</v>
+        <v>2.02</v>
       </c>
       <c r="S25">
-        <v>1.906</v>
+        <v>1.82</v>
       </c>
       <c r="T25">
-        <v>-1.516</v>
+        <v>0.5</v>
       </c>
       <c r="U25">
-        <v>1.964</v>
+        <v>2.02</v>
       </c>
       <c r="V25">
-        <v>1.879</v>
+        <v>1.82</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
@@ -11167,7 +11167,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:23.000Z</t>
+          <t>2026-05-23T13:58:54.000Z</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -11176,13 +11176,13 @@
         </is>
       </c>
       <c r="H26">
-        <v>3.354</v>
+        <v>3.272</v>
       </c>
       <c r="I26">
-        <v>3.562</v>
+        <v>3.534</v>
       </c>
       <c r="J26">
-        <v>2.097</v>
+        <v>2.138</v>
       </c>
       <c r="K26">
         <v>3.709</v>
@@ -11194,13 +11194,13 @@
         <v>1.883</v>
       </c>
       <c r="N26">
-        <v>0.355</v>
+        <v>0.437</v>
       </c>
       <c r="O26">
-        <v>0.293</v>
+        <v>0.321</v>
       </c>
       <c r="P26">
-        <v>-0.214</v>
+        <v>-0.255</v>
       </c>
       <c r="Q26">
         <v>0.516</v>
@@ -11212,13 +11212,13 @@
         <v>1.896</v>
       </c>
       <c r="T26">
-        <v>0.313</v>
+        <v>0.281</v>
       </c>
       <c r="U26">
-        <v>1.949</v>
+        <v>1.958</v>
       </c>
       <c r="V26">
-        <v>1.909</v>
+        <v>1.833</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
@@ -11279,7 +11279,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:30.000Z</t>
+          <t>2026-05-23T13:59:03.000Z</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -11288,13 +11288,13 @@
         </is>
       </c>
       <c r="H27">
-        <v>1.711</v>
+        <v>1.718</v>
       </c>
       <c r="I27">
-        <v>3.822</v>
+        <v>3.803</v>
       </c>
       <c r="J27">
-        <v>4.747</v>
+        <v>4.727</v>
       </c>
       <c r="K27">
         <v>1.491</v>
@@ -11306,13 +11306,13 @@
         <v>6.101</v>
       </c>
       <c r="N27">
-        <v>-0.22</v>
+        <v>-0.227</v>
       </c>
       <c r="O27">
-        <v>0.433</v>
+        <v>0.452</v>
       </c>
       <c r="P27">
-        <v>1.354</v>
+        <v>1.374</v>
       </c>
       <c r="Q27">
         <v>-1.062</v>
@@ -11327,10 +11327,10 @@
         <v>-0.719</v>
       </c>
       <c r="U27">
-        <v>1.895</v>
+        <v>1.918</v>
       </c>
       <c r="V27">
-        <v>1.951</v>
+        <v>1.929</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
@@ -11391,7 +11391,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:31.000Z</t>
+          <t>2026-05-23T13:59:04.000Z</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -11503,7 +11503,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:31.000Z</t>
+          <t>2026-05-23T14:00:53.683Z</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -11539,22 +11539,22 @@
         <v>0.343</v>
       </c>
       <c r="Q29">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="R29">
-        <v>1.879</v>
+        <v>1.98</v>
       </c>
       <c r="S29">
-        <v>1.795</v>
+        <v>1.88</v>
       </c>
       <c r="T29">
-        <v>-0.047</v>
+        <v>-0.5</v>
       </c>
       <c r="U29">
-        <v>1.821</v>
+        <v>1.98</v>
       </c>
       <c r="V29">
-        <v>1.989</v>
+        <v>1.88</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
@@ -11615,7 +11615,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:31.000Z</t>
+          <t>2026-05-23T13:59:04.000Z</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -11624,13 +11624,13 @@
         </is>
       </c>
       <c r="H30">
-        <v>1.812</v>
+        <v>1.813</v>
       </c>
       <c r="I30">
-        <v>3.863</v>
+        <v>3.86</v>
       </c>
       <c r="J30">
-        <v>4.063</v>
+        <v>4.06</v>
       </c>
       <c r="K30">
         <v>1.831</v>
@@ -11642,13 +11642,13 @@
         <v>3.888</v>
       </c>
       <c r="N30">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
       <c r="O30">
-        <v>-0.121</v>
+        <v>-0.118</v>
       </c>
       <c r="P30">
-        <v>-0.175</v>
+        <v>-0.172</v>
       </c>
       <c r="Q30">
         <v>-0.562</v>
@@ -11663,7 +11663,7 @@
         <v>-0.578</v>
       </c>
       <c r="U30">
-        <v>1.888</v>
+        <v>1.887</v>
       </c>
       <c r="V30">
         <v>1.958</v>
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:31.000Z</t>
+          <t>2026-05-23T13:59:04.000Z</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -11736,13 +11736,13 @@
         </is>
       </c>
       <c r="H31">
-        <v>2.291</v>
+        <v>2.31</v>
       </c>
       <c r="I31">
-        <v>3.423</v>
+        <v>3.421</v>
       </c>
       <c r="J31">
-        <v>3.066</v>
+        <v>3.036</v>
       </c>
       <c r="K31">
         <v>2.04</v>
@@ -11754,13 +11754,13 @@
         <v>3.285</v>
       </c>
       <c r="N31">
-        <v>-0.251</v>
+        <v>-0.27</v>
       </c>
       <c r="O31">
-        <v>0.281</v>
+        <v>0.283</v>
       </c>
       <c r="P31">
-        <v>0.219</v>
+        <v>0.249</v>
       </c>
       <c r="Q31">
         <v>-0.383</v>
@@ -11775,10 +11775,10 @@
         <v>-0.25</v>
       </c>
       <c r="U31">
-        <v>1.934</v>
+        <v>2.02</v>
       </c>
       <c r="V31">
-        <v>1.862</v>
+        <v>1.846</v>
       </c>
       <c r="W31" t="inlineStr">
         <is>
@@ -11839,7 +11839,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:14.000Z</t>
+          <t>2026-05-23T13:58:43.000Z</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -11848,13 +11848,13 @@
         </is>
       </c>
       <c r="H32">
-        <v>2.195</v>
+        <v>2.192</v>
       </c>
       <c r="I32">
-        <v>3.531</v>
+        <v>3.537</v>
       </c>
       <c r="J32">
-        <v>2.975</v>
+        <v>2.969</v>
       </c>
       <c r="K32">
         <v>2.303</v>
@@ -11866,13 +11866,13 @@
         <v>2.804</v>
       </c>
       <c r="N32">
-        <v>0.108</v>
+        <v>0.111</v>
       </c>
       <c r="O32">
-        <v>-0.142</v>
+        <v>-0.148</v>
       </c>
       <c r="P32">
-        <v>-0.171</v>
+        <v>-0.165</v>
       </c>
       <c r="Q32">
         <v>-0.094</v>
@@ -11887,10 +11887,10 @@
         <v>-0.281</v>
       </c>
       <c r="U32">
-        <v>1.964</v>
+        <v>1.952</v>
       </c>
       <c r="V32">
-        <v>1.859</v>
+        <v>1.892</v>
       </c>
       <c r="W32" t="inlineStr">
         <is>
@@ -11951,7 +11951,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:00.000Z</t>
+          <t>2026-05-23T14:00:52.588Z</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -11987,22 +11987,22 @@
         <v>-0.296</v>
       </c>
       <c r="Q33">
-        <v>-0.267</v>
+        <v>-0.5</v>
       </c>
       <c r="R33">
-        <v>1.858</v>
+        <v>2.1</v>
       </c>
       <c r="S33">
-        <v>1.957</v>
+        <v>1.7</v>
       </c>
       <c r="T33">
-        <v>-0.483</v>
+        <v>-0.5</v>
       </c>
       <c r="U33">
-        <v>1.999</v>
+        <v>2.1</v>
       </c>
       <c r="V33">
-        <v>1.837</v>
+        <v>1.7</v>
       </c>
       <c r="W33" t="inlineStr">
         <is>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:00.000Z</t>
+          <t>2026-05-23T14:00:52.587Z</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -12099,22 +12099,22 @@
         <v>-0.534</v>
       </c>
       <c r="Q34">
-        <v>-0.406</v>
+        <v>-0.75</v>
       </c>
       <c r="R34">
-        <v>1.936</v>
+        <v>2.1</v>
       </c>
       <c r="S34">
-        <v>1.872</v>
+        <v>1.7</v>
       </c>
       <c r="T34">
-        <v>-0.5</v>
+        <v>-0.75</v>
       </c>
       <c r="U34">
-        <v>1.904</v>
+        <v>2.1</v>
       </c>
       <c r="V34">
-        <v>1.86</v>
+        <v>1.7</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:07.000Z</t>
+          <t>2026-05-23T13:58:37.000Z</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -12187,10 +12187,10 @@
         <v>2.076</v>
       </c>
       <c r="I35">
-        <v>3.54</v>
+        <v>3.538</v>
       </c>
       <c r="J35">
-        <v>3.158</v>
+        <v>3.159</v>
       </c>
       <c r="K35">
         <v>1.778</v>
@@ -12205,10 +12205,10 @@
         <v>-0.298</v>
       </c>
       <c r="O35">
-        <v>0.307</v>
+        <v>0.309</v>
       </c>
       <c r="P35">
-        <v>0.732</v>
+        <v>0.731</v>
       </c>
       <c r="Q35">
         <v>-0.583</v>
@@ -12223,10 +12223,10 @@
         <v>-0.283</v>
       </c>
       <c r="U35">
-        <v>1.878</v>
+        <v>1.875</v>
       </c>
       <c r="V35">
-        <v>1.94</v>
+        <v>1.948</v>
       </c>
       <c r="W35" t="inlineStr">
         <is>
@@ -12287,7 +12287,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:08.000Z</t>
+          <t>2026-05-23T13:58:37.000Z</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -12296,13 +12296,13 @@
         </is>
       </c>
       <c r="H36">
-        <v>1.881</v>
+        <v>1.852</v>
       </c>
       <c r="I36">
-        <v>3.469</v>
+        <v>3.502</v>
       </c>
       <c r="J36">
-        <v>3.87</v>
+        <v>3.948</v>
       </c>
       <c r="K36">
         <v>1.866</v>
@@ -12314,13 +12314,13 @@
         <v>3.763</v>
       </c>
       <c r="N36">
-        <v>-0.015</v>
+        <v>0.014</v>
       </c>
       <c r="O36">
-        <v>0.017</v>
+        <v>-0.016</v>
       </c>
       <c r="P36">
-        <v>-0.107</v>
+        <v>-0.185</v>
       </c>
       <c r="Q36">
         <v>-0.533</v>
@@ -12335,10 +12335,10 @@
         <v>-0.517</v>
       </c>
       <c r="U36">
-        <v>1.921</v>
+        <v>1.901</v>
       </c>
       <c r="V36">
-        <v>1.896</v>
+        <v>1.928</v>
       </c>
       <c r="W36" t="inlineStr">
         <is>
@@ -12399,7 +12399,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:08.000Z</t>
+          <t>2026-05-23T13:58:38.000Z</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -12408,13 +12408,13 @@
         </is>
       </c>
       <c r="H37">
-        <v>1.536</v>
+        <v>1.507</v>
       </c>
       <c r="I37">
-        <v>3.955</v>
+        <v>4.057</v>
       </c>
       <c r="J37">
-        <v>5.74</v>
+        <v>5.934</v>
       </c>
       <c r="K37">
         <v>1.591</v>
@@ -12426,13 +12426,13 @@
         <v>5.063</v>
       </c>
       <c r="N37">
-        <v>0.055</v>
+        <v>0.084</v>
       </c>
       <c r="O37">
-        <v>-0.187</v>
+        <v>-0.289</v>
       </c>
       <c r="P37">
-        <v>-0.677</v>
+        <v>-0.871</v>
       </c>
       <c r="Q37">
         <v>-0.875</v>
@@ -12447,10 +12447,10 @@
         <v>-0.969</v>
       </c>
       <c r="U37">
-        <v>1.889</v>
+        <v>1.878</v>
       </c>
       <c r="V37">
-        <v>1.871</v>
+        <v>1.884</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-05-23T13:25:08.000Z</t>
+          <t>2026-05-23T13:58:38.000Z</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -12520,10 +12520,10 @@
         </is>
       </c>
       <c r="H38">
-        <v>2.402</v>
+        <v>2.391</v>
       </c>
       <c r="I38">
-        <v>3.435</v>
+        <v>3.468</v>
       </c>
       <c r="J38">
         <v>2.688</v>
@@ -12538,10 +12538,10 @@
         <v>2.532</v>
       </c>
       <c r="N38">
-        <v>0.082</v>
+        <v>0.093</v>
       </c>
       <c r="O38">
-        <v>-0.026</v>
+        <v>-0.059</v>
       </c>
       <c r="P38">
         <v>-0.156</v>
@@ -12556,13 +12556,13 @@
         <v>1.847</v>
       </c>
       <c r="T38">
-        <v>0</v>
+        <v>0.016</v>
       </c>
       <c r="U38">
-        <v>1.819</v>
+        <v>1.804</v>
       </c>
       <c r="V38">
-        <v>1.946</v>
+        <v>1.964</v>
       </c>
       <c r="W38" t="inlineStr">
         <is>
@@ -12899,7 +12899,7 @@
         </is>
       </c>
       <c r="G6">
-        <v>48.14</v>
+        <v>46.74</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -12949,7 +12949,7 @@
         </is>
       </c>
       <c r="G7">
-        <v>43.27</v>
+        <v>36.66</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -12958,7 +12958,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>主方向概率领先</t>
+          <t>备选赔付不高，市场不排除</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -13249,7 +13249,7 @@
         </is>
       </c>
       <c r="G13">
-        <v>35.91</v>
+        <v>31.71</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -13349,7 +13349,7 @@
         </is>
       </c>
       <c r="G15">
-        <v>20.86</v>
+        <v>16.66</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -13449,7 +13449,7 @@
         </is>
       </c>
       <c r="G17">
-        <v>30.97</v>
+        <v>26.77</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -13749,7 +13749,7 @@
         </is>
       </c>
       <c r="G23">
-        <v>65.26</v>
+        <v>61.06</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -13949,7 +13949,7 @@
         </is>
       </c>
       <c r="G27">
-        <v>43.27</v>
+        <v>36.66</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -14099,7 +14099,7 @@
         </is>
       </c>
       <c r="G30">
-        <v>20.86</v>
+        <v>16.66</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>

</xml_diff>